<commit_message>
Update project configurations and clean up gitignore
</commit_message>
<xml_diff>
--- a/UserData/UserData.xlsx
+++ b/UserData/UserData.xlsx
@@ -1,13 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{8B1666A9-4E20-412B-993A-775FD03299DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="MutualFound" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="Shares" sheetId="2" r:id="rId6"/>
+    <sheet name="MutualFound" sheetId="1" r:id="rId1"/>
+    <sheet name="Shares" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1"/>
 </workbook>
 </file>
 
@@ -67,10 +72,10 @@
   <si>
     <r>
       <rPr>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
         <rFont val="&quot;Aptos Narrow&quot;, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
       </rPr>
       <t>testvaluenable@gmail.com</t>
     </r>
@@ -117,10 +122,10 @@
   <si>
     <r>
       <rPr>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
         <rFont val="&quot;Aptos Narrow&quot;, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
       </rPr>
       <t>testvaluenable@gmail.com</t>
     </r>
@@ -135,53 +140,59 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="mm-dd-yyyy"/>
+    <numFmt numFmtId="164" formatCode="mm\-dd\-yyyy"/>
   </numFmts>
-  <fonts count="8">
-    <font>
-      <sz val="10.0"/>
+  <fonts count="9">
+    <font>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="&quot;Aptos Narrow&quot;"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Consolas"/>
     </font>
     <font>
       <u/>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="&quot;Aptos Narrow&quot;"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF3F7F5F"/>
       <name val="&quot;Aptos Narrow&quot;"/>
     </font>
     <font>
-      <sz val="8.0"/>
+      <sz val="8"/>
       <color rgb="FF2A00FF"/>
       <name val="Consolas"/>
     </font>
     <font>
       <u/>
-      <sz val="8.0"/>
+      <sz val="8"/>
       <color rgb="FF3F7F5F"/>
       <name val="Consolas"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF1155CC"/>
+      <name val="&quot;Aptos Narrow&quot;, sans-serif"/>
     </font>
   </fonts>
   <fills count="2">
@@ -189,71 +200,58 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="11">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -443,20 +441,23 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="14" max="14" width="20.0"/>
+    <col min="14" max="14" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:15" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -503,12 +504,12 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:15">
       <c r="A2" s="3">
-        <v>9.999999951E9</v>
+        <v>9999999951</v>
       </c>
       <c r="B2" s="3">
-        <v>100000.0</v>
+        <v>100000</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>15</v>
@@ -520,10 +521,10 @@
         <v>17</v>
       </c>
       <c r="F2" s="5">
-        <v>37715.0</v>
+        <v>37715</v>
       </c>
       <c r="G2" s="3">
-        <v>3000000.0</v>
+        <v>100000</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>18</v>
@@ -552,28 +553,29 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="E2"/>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
   </hyperlinks>
-  <drawing r:id="rId2"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:T2"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="4" max="4" width="18.25"/>
-    <col customWidth="1" min="5" max="5" width="23.0"/>
-    <col customWidth="1" min="10" max="10" width="13.0"/>
-    <col customWidth="1" min="11" max="11" width="15.63"/>
-    <col customWidth="1" min="17" max="17" width="15.0"/>
-    <col customWidth="1" min="19" max="19" width="20.0"/>
+    <col min="4" max="4" width="18.21875" customWidth="1"/>
+    <col min="5" max="5" width="23" customWidth="1"/>
+    <col min="10" max="10" width="13" customWidth="1"/>
+    <col min="11" max="11" width="15.6640625" customWidth="1"/>
+    <col min="17" max="17" width="15" customWidth="1"/>
+    <col min="19" max="19" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:20" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -635,12 +637,12 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:20">
       <c r="A2" s="3">
-        <v>9.999999951E9</v>
+        <v>9999999951</v>
       </c>
       <c r="B2" s="3">
-        <v>100000.0</v>
+        <v>100000</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>15</v>
@@ -652,16 +654,16 @@
         <v>31</v>
       </c>
       <c r="F2" s="5">
-        <v>37715.0</v>
+        <v>37715</v>
       </c>
       <c r="G2" s="3">
-        <v>3000000.0</v>
+        <v>3000000</v>
       </c>
       <c r="H2" s="3">
-        <v>1.2000012E7</v>
+        <v>12000012</v>
       </c>
       <c r="I2" s="8">
-        <v>1.2000012E7</v>
+        <v>12000012</v>
       </c>
       <c r="J2" s="9" t="s">
         <v>32</v>
@@ -670,7 +672,7 @@
         <v>33</v>
       </c>
       <c r="L2" s="8">
-        <v>200.0</v>
+        <v>200</v>
       </c>
       <c r="M2" s="1" t="s">
         <v>18</v>
@@ -699,8 +701,8 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="E2"/>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
   </hyperlinks>
-  <drawing r:id="rId2"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>